<commit_message>
feat(source): surface signal-stage contract levers
</commit_message>
<xml_diff>
--- a/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
+++ b/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb76c96a02a54430b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="Rb5d83f3afb2e49da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="R9ce0f5f1d362438a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="R525728aa26b74e39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R1bc7bbceb50744d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="Ra27f352bf2d24ab7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R304cd50f331d4e98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="Rb4ca76f11ca14b34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="R649ec8cd3b1d41b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="R58375f508aa5430e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R3d6345de008e4246"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R4e0e28510a7042d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -395,7 +395,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcd962e683e5a4e96"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R25f6d76c667541d0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -779,7 +779,7 @@
         <x:v>Candidate annual opportunity</x:v>
       </x:c>
       <x:c r="B11" s="20" t="n">
-        <x:v>1511000</x:v>
+        <x:v>1836000</x:v>
       </x:c>
       <x:c r="C11" s="17"/>
       <x:c r="D11" s="17" t="str">
@@ -882,7 +882,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff5cdc03af3d4fa0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfed0d215d5c646b3"/>
 </x:worksheet>
 </file>
 
@@ -1190,7 +1190,7 @@
     <x:col min="3" max="3" width="6.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="5.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="34.66999816894531" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="52.11000061035156" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="76.11000061035156" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="127.88999938964844" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -1327,6 +1327,52 @@
       </x:c>
       <x:c r="G8" s="17" t="str">
         <x:v>clause:MER-TECH-DBX-001:marketplace_routing;cloud_account:AWS-PAYER-001;commitment:DBX-COMMIT-2025-Y1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="17" t="str">
+        <x:v>Signal-stage discount band re-price review</x:v>
+      </x:c>
+      <x:c r="B9" s="20" t="n">
+        <x:v>150000</x:v>
+      </x:c>
+      <x:c r="C9" s="20" t="n">
+        <x:v>450000</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="E9" s="17" t="str">
+        <x:v>Strategic Sourcing with Technology Finance</x:v>
+      </x:c>
+      <x:c r="F9" s="17" t="str">
+        <x:v>Treat as advisory until a comparable benchmark is loaded; request re-pricing evidence for the five-year volume tier.</x:v>
+      </x:c>
+      <x:c r="G9" s="17" t="str">
+        <x:v>clause:MER-TECH-DBX-001:benchmarking_clause;clause:MER-TECH-DBX-001:minimum_commitment;commitment:DBX-COMMIT-2025-Y1;DOC-MER-TECH-DBX-001-ORDER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="17" t="str">
+        <x:v>Signal-stage serverless/classic discount parity check</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="n">
+        <x:v>80000</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="E10" s="17" t="str">
+        <x:v>Cloud FinOps and Enterprise Data Platforms</x:v>
+      </x:c>
+      <x:c r="F10" s="17" t="str">
+        <x:v>Confirm discount parity and per-SKU economics before shifting bursty pilot jobs from classic compute to serverless.</x:v>
+      </x:c>
+      <x:c r="G10" s="17" t="str">
+        <x:v>cloud_usage:MER-TECH-DBX-001:2026-08:JOBS-COMPUTE;cloud_usage:MER-TECH-DBX-001:2026-09:JOBS-COMPUTE;DOC-MER-TECH-DBX-001-USAGE</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1618,6 +1664,142 @@
       </x:c>
       <x:c r="B38" s="17" t="str">
         <x:v>clause:MER-TECH-DBX-001:marketplace_routing;cloud_account:AWS-PAYER-001;commitment:DBX-COMMIT-2025-Y1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="A39" s="17"/>
+      <x:c r="B39" s="17"/>
+    </x:row>
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
+      <x:c r="A40" s="24" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="B40" s="24" t="str">
+        <x:v>Signal-stage discount band re-price review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="15" hidden="0" customHeight="1">
+      <x:c r="A41" s="18" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="B41" s="17" t="str">
+        <x:v>Strategic Sourcing with Technology Finance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="18" t="str">
+        <x:v>Buyer ask</x:v>
+      </x:c>
+      <x:c r="B42" s="17" t="str">
+        <x:v>Re-price the platform services discount band after Finance loads an accepted comparable for a similar multi-year consumption-platform commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="18" t="str">
+        <x:v>Negotiation language</x:v>
+      </x:c>
+      <x:c r="B43" s="17" t="str">
+        <x:v>This is an advisory signal, not a document-proven finding. The current package shows the commitment size and confirms benchmarking is absent, so we are asking Databricks to re-open discount-band evidence once a comparable five-year volume benchmark is available.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="18" t="str">
+        <x:v>Vendor concession</x:v>
+      </x:c>
+      <x:c r="B44" s="17" t="str">
+        <x:v>Databricks would move from the current discount position to a benchmark-supported tier if the buyer proves comparable market terms.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="18" t="str">
+        <x:v>Timing dependency</x:v>
+      </x:c>
+      <x:c r="B45" s="17" t="str">
+        <x:v>Load one accepted benchmark comparable before treating this as an executive ask in the Year 2 amendment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="18" t="str">
+        <x:v>Risk if ignored</x:v>
+      </x:c>
+      <x:c r="B46" s="17" t="str">
+        <x:v>The buyer may negotiate only ramp timing and credits while leaving a potentially mispriced discount band untested.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
+      <x:c r="A47" s="18" t="str">
+        <x:v>Evidence rows</x:v>
+      </x:c>
+      <x:c r="B47" s="17" t="str">
+        <x:v>clause:MER-TECH-DBX-001:benchmarking_clause;clause:MER-TECH-DBX-001:minimum_commitment;commitment:DBX-COMMIT-2025-Y1;DOC-MER-TECH-DBX-001-ORDER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="A48" s="17"/>
+      <x:c r="B48" s="17"/>
+    </x:row>
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="A49" s="24" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="B49" s="24" t="str">
+        <x:v>Signal-stage serverless/classic discount parity check</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="A50" s="18" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="B50" s="17" t="str">
+        <x:v>Cloud FinOps and Enterprise Data Platforms</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="A51" s="18" t="str">
+        <x:v>Buyer ask</x:v>
+      </x:c>
+      <x:c r="B51" s="17" t="str">
+        <x:v>Confirm committed-discount treatment across serverless and classic compute and load a side-by-side per-SKU cost comparison before workload migration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="18" t="str">
+        <x:v>Negotiation language</x:v>
+      </x:c>
+      <x:c r="B52" s="17" t="str">
+        <x:v>This is a workload-shape signal, not a priced finding. The package shows bursty pilot jobs-compute usage, but it does not include per-SKU serverless comparison evidence, so the ask is to confirm discount parity before making serverless the default operating model.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="18" t="str">
+        <x:v>Vendor concession</x:v>
+      </x:c>
+      <x:c r="B53" s="17" t="str">
+        <x:v>Databricks would preserve committed-discount economics across the target compute mode or provide a clear commercial bridge for the migrated workload.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="18" t="str">
+        <x:v>Timing dependency</x:v>
+      </x:c>
+      <x:c r="B54" s="17" t="str">
+        <x:v>Complete before the pilot workload moves from classic jobs compute into production serverless jobs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="A55" s="18" t="str">
+        <x:v>Risk if ignored</x:v>
+      </x:c>
+      <x:c r="B55" s="17" t="str">
+        <x:v>A technically sensible compute shift could dilute the committed discount or move spend into a SKU pattern the contract does not protect.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
+      <x:c r="A56" s="18" t="str">
+        <x:v>Evidence rows</x:v>
+      </x:c>
+      <x:c r="B56" s="17" t="str">
+        <x:v>cloud_usage:MER-TECH-DBX-001:2026-08:JOBS-COMPUTE;cloud_usage:MER-TECH-DBX-001:2026-09:JOBS-COMPUTE;DOC-MER-TECH-DBX-001-USAGE</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2023,10 +2205,10 @@
         <x:v>Opportunities not finance-confirmed</x:v>
       </x:c>
       <x:c r="B11" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C11" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D11" s="17" t="str">
         <x:v>PASS</x:v>

</xml_diff>

<commit_message>
fix(source): require reviewed contract context
</commit_message>
<xml_diff>
--- a/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
+++ b/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R304cd50f331d4e98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="Rb4ca76f11ca14b34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="R649ec8cd3b1d41b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="R58375f508aa5430e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R3d6345de008e4246"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R4e0e28510a7042d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3040f58b283b453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="R84615ea3d7bd4ea6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="Rbd057b9cecea450a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="Rb1656e44c13b47d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rfa3caeb752c146fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R612f9241396549ae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -395,7 +395,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R25f6d76c667541d0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6c43286872cc4881"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -882,7 +882,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfed0d215d5c646b3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfde451f52d7448d"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix(source): protect document ownership boundaries
</commit_message>
<xml_diff>
--- a/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
+++ b/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3040f58b283b453b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="R84615ea3d7bd4ea6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="Rbd057b9cecea450a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="Rb1656e44c13b47d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rfa3caeb752c146fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R612f9241396549ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra12902ed6cfd4f95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="Rb316df8b43614819"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="R3ea1ff2e299f4b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="Rd93b1e25fcd6482e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Ra3f03fa6d2d34fc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R79a7a88a61d44c79"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -395,7 +395,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6c43286872cc4881"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf1dd9d5263fd4daa"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -882,7 +882,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfde451f52d7448d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b3552be735d4dcb"/>
 </x:worksheet>
 </file>
 
@@ -1813,7 +1813,7 @@
   <x:cols>
     <x:col min="1" max="1" width="13.109999656677246" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="36.66999816894531" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="26.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14.779999732971191" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="17.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="10.670000076293945" hidden="0" customWidth="1"/>
@@ -2049,7 +2049,7 @@
         <x:v>meridian-databricks-consumption-commit-v1-20260908</x:v>
       </x:c>
       <x:c r="C10" s="17" t="str">
-        <x:v>DOC-MER-CLOUD-AWS-001-EDP</x:v>
+        <x:v>DOC-MER-TECH-DBX-001-AWS-MARKETPLACE</x:v>
       </x:c>
       <x:c r="D10" s="17" t="str">
         <x:v>MER-TECH-DBX-001</x:v>

</xml_diff>

<commit_message>
Protect Source document ownership boundaries (#7633)
* Add governed Source projection refresh entrypoints

* fix source document evidence retries

* docs: name source data release lane

* fix(source): protect document ownership boundaries

---------

Co-authored-by: Anand Sundaram <anandsundaram-hash@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
+++ b/datasets/source/cloud-consumption/meridian-databricks-consumption-commit-v1-20260908/Meridian_Databricks_Consumption_Commit_Intake_Workbook_v1.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3040f58b283b453b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="R84615ea3d7bd4ea6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="Rbd057b9cecea450a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="Rb1656e44c13b47d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rfa3caeb752c146fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R612f9241396549ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra12902ed6cfd4f95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" r:id="Rb316df8b43614819"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" r:id="R3ea1ff2e299f4b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levers" sheetId="4" r:id="Rd93b1e25fcd6482e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Ra3f03fa6d2d34fc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R79a7a88a61d44c79"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -395,7 +395,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6c43286872cc4881"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf1dd9d5263fd4daa"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -882,7 +882,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfde451f52d7448d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b3552be735d4dcb"/>
 </x:worksheet>
 </file>
 
@@ -1813,7 +1813,7 @@
   <x:cols>
     <x:col min="1" max="1" width="13.109999656677246" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="36.66999816894531" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="26.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14.779999732971191" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="17.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="10.670000076293945" hidden="0" customWidth="1"/>
@@ -2049,7 +2049,7 @@
         <x:v>meridian-databricks-consumption-commit-v1-20260908</x:v>
       </x:c>
       <x:c r="C10" s="17" t="str">
-        <x:v>DOC-MER-CLOUD-AWS-001-EDP</x:v>
+        <x:v>DOC-MER-TECH-DBX-001-AWS-MARKETPLACE</x:v>
       </x:c>
       <x:c r="D10" s="17" t="str">
         <x:v>MER-TECH-DBX-001</x:v>

</xml_diff>